<commit_message>
Enriquecer patrones: 600+ medicamentos, limpieza y gases adicionales
</commit_message>
<xml_diff>
--- a/resultados_v5/resumen_clasificacion_avanzada.xlsx
+++ b/resultados_v5/resumen_clasificacion_avanzada.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,17 +429,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Clasificación</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Confianza Promedio</t>
         </is>
@@ -440,7 +452,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>83675</v>
+        <v>16699</v>
       </c>
       <c r="C2" t="n">
         <v>0.95</v>
@@ -453,7 +465,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>35273</v>
+        <v>7131</v>
       </c>
       <c r="C3" t="n">
         <v>0.95</v>
@@ -466,7 +478,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5836</v>
+        <v>1101</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
@@ -479,10 +491,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4893</v>
+        <v>988</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9499999999999998</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="6">
@@ -492,10 +504,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3973</v>
+        <v>803</v>
       </c>
       <c r="C6" t="n">
-        <v>0.95</v>
+        <v>0.9499999999999998</v>
       </c>
     </row>
     <row r="7">
@@ -505,7 +517,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3711</v>
+        <v>747</v>
       </c>
       <c r="C7" t="n">
         <v>0.95</v>
@@ -518,10 +530,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3333</v>
+        <v>648</v>
       </c>
       <c r="C8" t="n">
-        <v>0.95</v>
+        <v>0.9500000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -531,7 +543,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1597</v>
+        <v>315</v>
       </c>
       <c r="C9" t="n">
         <v>0.95</v>
@@ -544,10 +556,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>866</v>
+        <v>177</v>
       </c>
       <c r="C10" t="n">
-        <v>0.95</v>
+        <v>0.9500000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -557,10 +569,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>625</v>
+        <v>142</v>
       </c>
       <c r="C11" t="n">
-        <v>0.95</v>
+        <v>0.9500000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -570,7 +582,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>376</v>
+        <v>80</v>
       </c>
       <c r="C12" t="n">
         <v>0.95</v>

</xml_diff>

<commit_message>
chore: baseline snapshot before next modifications
</commit_message>
<xml_diff>
--- a/resultados_v5/resumen_clasificacion_avanzada.xlsx
+++ b/resultados_v5/resumen_clasificacion_avanzada.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,167 +425,864 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clasificación</t>
+          <t>origen_hoja</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>grupo_sustancia_final</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Confianza Promedio</t>
+          <t>conteo</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>356_2022</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>otros</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>16699</v>
-      </c>
       <c r="C2" t="n">
-        <v>0.95</v>
+        <v>21328</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>tranquilizantes_y_sedantes</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>7131</v>
+          <t>356_2022</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>medicamentos_no_SPA</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>0.95</v>
+        <v>12394</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AGRO_PRODUCT</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1101</v>
+          <t>356_2022</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>tranquilizantes_y_sedantes</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>7594</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>alcohol_etanol</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>988</v>
+          <t>356_2022</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>opioides</t>
+        </is>
       </c>
       <c r="C5" t="n">
-        <v>0.95</v>
+        <v>774</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>cannabinoides</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>803</v>
+          <t>356_2022</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>productos_limpieza</t>
+        </is>
       </c>
       <c r="C6" t="n">
-        <v>0.9499999999999998</v>
+        <v>221</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>opioides</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>747</v>
+          <t>356_2022</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>alcohol_etanol</t>
+        </is>
       </c>
       <c r="C7" t="n">
-        <v>0.95</v>
+        <v>198</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>356_2022</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>cocaina_y_derivados</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>648</v>
-      </c>
       <c r="C8" t="n">
-        <v>0.9500000000000001</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>inhalantes</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>315</v>
+          <t>356_2022</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>gases_combustibles</t>
+        </is>
       </c>
       <c r="C9" t="n">
-        <v>0.95</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>escopolamina</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>177</v>
+          <t>356_2022</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>cannabinoides</t>
+        </is>
       </c>
       <c r="C10" t="n">
-        <v>0.9500000000000001</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>356_2022</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>alucinogenos</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>142</v>
-      </c>
       <c r="C11" t="n">
-        <v>0.9500000000000001</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>356_2022</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>estimulantes</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>80</v>
-      </c>
       <c r="C12" t="n">
-        <v>0.95</v>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>356_2022</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>inhalantes</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>356_2022</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>escopolamina</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>356_2022</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PSA_no_clasificado_lista</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>356_2023</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>otros</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>23510</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>356_2023</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>medicamentos_no_SPA</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>13273</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>356_2023</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>tranquilizantes_y_sedantes</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>8665</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>356_2023</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>opioides</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>356_2023</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>productos_limpieza</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>356_2023</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>alcohol_etanol</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>356_2023</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>cocaina_y_derivados</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>356_2023</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>gases_combustibles</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>356_2023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>alucinogenos</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>356_2023</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>cannabinoides</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>356_2023</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>estimulantes</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>356_2023</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>inhalantes</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>356_2023</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>escopolamina</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>356_2023</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PSA_no_clasificado_lista</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>365_2022</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>otros</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>18176</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>365_2022</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>medicamentos_no_SPA</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>14467</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>365_2022</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>tranquilizantes_y_sedantes</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>8854</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>365_2022</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>alcohol_etanol</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2425</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>365_2022</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>cannabinoides</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1883</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>365_2022</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>cocaina_y_derivados</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1634</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>365_2022</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>opioides</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1131</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>365_2022</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>productos_limpieza</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>365_2022</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>escopolamina</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>365_2022</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>gases_combustibles</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>365_2022</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>alucinogenos</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>365_2022</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>inhalantes</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>365_2022</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>estimulantes</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>365_2022</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>PSA_no_clasificado_lista</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>365_2023</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>otros</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>20616</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>365_2023</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>medicamentos_no_SPA</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>15148</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>365_2023</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>tranquilizantes_y_sedantes</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>10101</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>365_2023</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>alcohol_etanol</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2252</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>365_2023</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>cannabinoides</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>1958</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>365_2023</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>cocaina_y_derivados</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>1568</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>365_2023</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>opioides</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>1193</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>365_2023</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>productos_limpieza</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>365_2023</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>gases_combustibles</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>365_2023</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>escopolamina</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>365_2023</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>alucinogenos</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>365_2023</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>estimulantes</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>365_2023</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>inhalantes</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>365_2023</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>PSA_no_clasificado_lista</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>